<commit_message>
power naar draw rename bij enemies voor duidelijkheid en verdere balance wijzigingen
</commit_message>
<xml_diff>
--- a/data/denizens_creature_database.xlsx
+++ b/data/denizens_creature_database.xlsx
@@ -3304,7 +3304,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
+    <row r="25" ht="57.6" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>C_GOBLIN_HEXER</t>
@@ -3331,7 +3331,7 @@
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -3349,10 +3349,10 @@
         <v>1</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>0</v>
@@ -3393,32 +3393,32 @@
       </c>
       <c r="Y25" s="6" t="inlineStr">
         <is>
-          <t>Hex Bolt — Ranged Magic Attack 2.</t>
+          <t>Hex Bolt — Ranged Attack 3.</t>
         </is>
       </c>
       <c r="Z25" s="6" t="inlineStr">
         <is>
-          <t>Crackling Hex — Ranged Magic Attack 3.</t>
+          <t>Crackling Hex — Ranged Attack 4.</t>
         </is>
       </c>
       <c r="AA25" s="6" t="inlineStr">
         <is>
-          <t>Jinx Guard — Remove 2 Guard from the target; if it has no Guard, Ranged Magic Attack 2 instead.</t>
+          <t>Jinx Guard — Attack 3, Sunder 2</t>
         </is>
       </c>
       <c r="AB25" s="6" t="inlineStr">
         <is>
-          <t>Scurrying Ward — Move 5 ft. One ally within 30 ft gains 2 Guard.</t>
+          <t>Scurrying Ward — One ally within 30 ft gains 5 Guard. While this Guard remains, any creature that hits the ally with a melee attack is lashed by the shield and suffers Attack 3.</t>
         </is>
       </c>
       <c r="AC25" s="6" t="inlineStr">
         <is>
-          <t>Bad Luck Charm — Ranged Magic Attack 3. The target cannot gain Guard until the start of the hexer’s next activation.</t>
+          <t>Bad Luck Charm — Ranged Magic Attack 4. The target cannot gain Guard until the start of the hexer’s next activation.</t>
         </is>
       </c>
       <c r="AD25" s="6" t="inlineStr">
         <is>
-          <t>Hex Burst — Ranged Magic Attack 5. If this deals a Wound, the target discards 1 random card from hand.</t>
+          <t>Hex Burst — Ranged Magic Attack 5, Shatter. If this deals a Wound, the target discards 1 random card from hand.</t>
         </is>
       </c>
       <c r="AE25" s="6" t="n"/>
@@ -3993,25 +3993,25 @@
         <v>2</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="M29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2</v>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="Y29" s="6" t="inlineStr">
         <is>
-          <t>Royal Jab — Attack 3.</t>
+          <t>Royal Jab — Attack 5.</t>
         </is>
       </c>
       <c r="Z29" s="6" t="inlineStr">
@@ -4047,12 +4047,12 @@
       </c>
       <c r="AA29" s="6" t="inlineStr">
         <is>
-          <t>Gang Command — Attack 3. If another goblin is adjacent to the target, Attack 5 instead.</t>
+          <t>Gang Command — Attack 4, Overwhelm.</t>
         </is>
       </c>
       <c r="AB29" s="6" t="inlineStr">
         <is>
-          <t>Scurry and Command — Move 5 ft. One goblin ally within 30 ft may Move 5 ft and Attack 2.</t>
+          <t>Scurry and Command — Gain 3 Guard. One goblin ally within 30 ft may Move 5 ft and Attack 2.</t>
         </is>
       </c>
       <c r="AC29" s="6" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="AD29" s="6" t="inlineStr">
         <is>
-          <t>Crown of Knives — Attack 5, Stab. Up to two goblin allies within 30 ft may each Move 5 ft.</t>
+          <t>Crown of Knives — Attack 5, Pierce 4. Up to two goblin allies within 30 ft may each Move 5 ft and Attack 2.</t>
         </is>
       </c>
       <c r="AE29" s="6" t="n"/>
@@ -5989,7 +5989,7 @@
       <c r="AG48" s="6" t="n"/>
       <c r="AH48" s="6" t="n"/>
       <c r="AI48" s="6" t="n"/>
-      <c r="AJ48" s="10" t="inlineStr"/>
+      <c r="AJ48" s="10" t="n"/>
       <c r="AK48" s="7" t="n"/>
       <c r="AL48" s="11" t="inlineStr">
         <is>
@@ -6078,7 +6078,7 @@
       <c r="AG49" s="6" t="n"/>
       <c r="AH49" s="6" t="n"/>
       <c r="AI49" s="6" t="n"/>
-      <c r="AJ49" s="10" t="inlineStr"/>
+      <c r="AJ49" s="10" t="n"/>
       <c r="AK49" s="7" t="n"/>
       <c r="AL49" s="11" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
       <c r="AG50" s="6" t="n"/>
       <c r="AH50" s="6" t="n"/>
       <c r="AI50" s="6" t="n"/>
-      <c r="AJ50" s="10" t="inlineStr"/>
+      <c r="AJ50" s="10" t="n"/>
       <c r="AK50" s="7" t="n"/>
       <c r="AL50" s="11" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
       <c r="AG51" s="6" t="n"/>
       <c r="AH51" s="6" t="n"/>
       <c r="AI51" s="6" t="n"/>
-      <c r="AJ51" s="10" t="inlineStr"/>
+      <c r="AJ51" s="10" t="n"/>
       <c r="AK51" s="7" t="n"/>
       <c r="AL51" s="11" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
       <c r="AG52" s="6" t="n"/>
       <c r="AH52" s="6" t="n"/>
       <c r="AI52" s="6" t="n"/>
-      <c r="AJ52" s="10" t="inlineStr"/>
+      <c r="AJ52" s="10" t="n"/>
       <c r="AK52" s="7" t="n"/>
       <c r="AL52" s="11" t="inlineStr">
         <is>
@@ -6434,7 +6434,7 @@
       <c r="AG53" s="6" t="n"/>
       <c r="AH53" s="6" t="n"/>
       <c r="AI53" s="6" t="n"/>
-      <c r="AJ53" s="10" t="inlineStr"/>
+      <c r="AJ53" s="10" t="n"/>
       <c r="AK53" s="7" t="n"/>
       <c r="AL53" s="11" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
       <c r="AG54" s="6" t="n"/>
       <c r="AH54" s="6" t="n"/>
       <c r="AI54" s="6" t="n"/>
-      <c r="AJ54" s="10" t="inlineStr"/>
+      <c r="AJ54" s="10" t="n"/>
       <c r="AK54" s="7" t="n"/>
       <c r="AL54" s="11" t="inlineStr">
         <is>
@@ -6612,7 +6612,7 @@
       <c r="AG55" s="6" t="n"/>
       <c r="AH55" s="6" t="n"/>
       <c r="AI55" s="6" t="n"/>
-      <c r="AJ55" s="10" t="inlineStr"/>
+      <c r="AJ55" s="10" t="n"/>
       <c r="AK55" s="7" t="n"/>
       <c r="AL55" s="11" t="inlineStr">
         <is>
@@ -6701,7 +6701,7 @@
       <c r="AG56" s="6" t="n"/>
       <c r="AH56" s="6" t="n"/>
       <c r="AI56" s="6" t="n"/>
-      <c r="AJ56" s="10" t="inlineStr"/>
+      <c r="AJ56" s="10" t="n"/>
       <c r="AK56" s="7" t="n"/>
       <c r="AL56" s="11" t="inlineStr">
         <is>
@@ -6790,7 +6790,7 @@
       <c r="AG57" s="6" t="n"/>
       <c r="AH57" s="6" t="n"/>
       <c r="AI57" s="6" t="n"/>
-      <c r="AJ57" s="10" t="inlineStr"/>
+      <c r="AJ57" s="10" t="n"/>
       <c r="AK57" s="7" t="n"/>
       <c r="AL57" s="11" t="inlineStr">
         <is>
@@ -10207,7 +10207,7 @@
       <c r="AG90" s="6" t="n"/>
       <c r="AH90" s="6" t="n"/>
       <c r="AI90" s="6" t="n"/>
-      <c r="AJ90" s="10" t="inlineStr"/>
+      <c r="AJ90" s="10" t="n"/>
       <c r="AK90" s="7" t="n"/>
       <c r="AL90" s="11" t="inlineStr">
         <is>
@@ -10296,7 +10296,7 @@
       <c r="AG91" s="6" t="n"/>
       <c r="AH91" s="6" t="n"/>
       <c r="AI91" s="6" t="n"/>
-      <c r="AJ91" s="10" t="inlineStr"/>
+      <c r="AJ91" s="10" t="n"/>
       <c r="AK91" s="7" t="n"/>
       <c r="AL91" s="11" t="inlineStr">
         <is>
@@ -10385,7 +10385,7 @@
       <c r="AG92" s="6" t="n"/>
       <c r="AH92" s="6" t="n"/>
       <c r="AI92" s="6" t="n"/>
-      <c r="AJ92" s="10" t="inlineStr"/>
+      <c r="AJ92" s="10" t="n"/>
       <c r="AK92" s="7" t="n"/>
       <c r="AL92" s="11" t="inlineStr">
         <is>
@@ -10474,7 +10474,7 @@
       <c r="AG93" s="6" t="n"/>
       <c r="AH93" s="6" t="n"/>
       <c r="AI93" s="6" t="n"/>
-      <c r="AJ93" s="10" t="inlineStr"/>
+      <c r="AJ93" s="10" t="n"/>
       <c r="AK93" s="7" t="n"/>
       <c r="AL93" s="11" t="inlineStr">
         <is>
@@ -10563,7 +10563,7 @@
       <c r="AG94" s="6" t="n"/>
       <c r="AH94" s="6" t="n"/>
       <c r="AI94" s="6" t="n"/>
-      <c r="AJ94" s="10" t="inlineStr"/>
+      <c r="AJ94" s="10" t="n"/>
       <c r="AK94" s="7" t="n"/>
       <c r="AL94" s="11" t="inlineStr">
         <is>
@@ -10652,7 +10652,7 @@
       <c r="AG95" s="6" t="n"/>
       <c r="AH95" s="6" t="n"/>
       <c r="AI95" s="6" t="n"/>
-      <c r="AJ95" s="10" t="inlineStr"/>
+      <c r="AJ95" s="10" t="n"/>
       <c r="AK95" s="7" t="n"/>
       <c r="AL95" s="11" t="inlineStr">
         <is>
@@ -14716,13 +14716,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ135" s="10" t="inlineStr"/>
+      <c r="AJ135" s="10" t="n"/>
       <c r="AK135" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL135" s="11" t="inlineStr"/>
+      <c r="AL135" s="11" t="n"/>
       <c r="AM135" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -22916,13 +22916,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ215" s="10" t="inlineStr"/>
+      <c r="AJ215" s="10" t="n"/>
       <c r="AK215" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL215" s="11" t="inlineStr"/>
+      <c r="AL215" s="11" t="n"/>
       <c r="AM215" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -23009,13 +23009,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ216" s="10" t="inlineStr"/>
+      <c r="AJ216" s="10" t="n"/>
       <c r="AK216" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL216" s="11" t="inlineStr"/>
+      <c r="AL216" s="11" t="n"/>
       <c r="AM216" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -23102,13 +23102,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ217" s="10" t="inlineStr"/>
+      <c r="AJ217" s="10" t="n"/>
       <c r="AK217" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL217" s="11" t="inlineStr"/>
+      <c r="AL217" s="11" t="n"/>
       <c r="AM217" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -23195,13 +23195,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ218" s="10" t="inlineStr"/>
+      <c r="AJ218" s="10" t="n"/>
       <c r="AK218" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL218" s="11" t="inlineStr"/>
+      <c r="AL218" s="11" t="n"/>
       <c r="AM218" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -23607,13 +23607,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ222" s="10" t="inlineStr"/>
+      <c r="AJ222" s="10" t="n"/>
       <c r="AK222" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL222" s="11" t="inlineStr"/>
+      <c r="AL222" s="11" t="n"/>
       <c r="AM222" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -23700,13 +23700,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ223" s="10" t="inlineStr"/>
+      <c r="AJ223" s="10" t="n"/>
       <c r="AK223" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL223" s="11" t="inlineStr"/>
+      <c r="AL223" s="11" t="n"/>
       <c r="AM223" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26103,13 +26103,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ246" s="10" t="inlineStr"/>
+      <c r="AJ246" s="10" t="n"/>
       <c r="AK246" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL246" s="11" t="inlineStr"/>
+      <c r="AL246" s="11" t="n"/>
       <c r="AM246" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26196,13 +26196,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ247" s="10" t="inlineStr"/>
+      <c r="AJ247" s="10" t="n"/>
       <c r="AK247" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL247" s="11" t="inlineStr"/>
+      <c r="AL247" s="11" t="n"/>
       <c r="AM247" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26289,13 +26289,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ248" s="10" t="inlineStr"/>
+      <c r="AJ248" s="10" t="n"/>
       <c r="AK248" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL248" s="11" t="inlineStr"/>
+      <c r="AL248" s="11" t="n"/>
       <c r="AM248" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26382,13 +26382,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ249" s="10" t="inlineStr"/>
+      <c r="AJ249" s="10" t="n"/>
       <c r="AK249" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL249" s="11" t="inlineStr"/>
+      <c r="AL249" s="11" t="n"/>
       <c r="AM249" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26475,13 +26475,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ250" s="10" t="inlineStr"/>
+      <c r="AJ250" s="10" t="n"/>
       <c r="AK250" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL250" s="11" t="inlineStr"/>
+      <c r="AL250" s="11" t="n"/>
       <c r="AM250" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26568,13 +26568,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ251" s="10" t="inlineStr"/>
+      <c r="AJ251" s="10" t="n"/>
       <c r="AK251" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL251" s="11" t="inlineStr"/>
+      <c r="AL251" s="11" t="n"/>
       <c r="AM251" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -26665,13 +26665,13 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ252" s="10" t="inlineStr"/>
+      <c r="AJ252" s="10" t="n"/>
       <c r="AK252" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL252" s="11" t="inlineStr"/>
+      <c r="AL252" s="11" t="n"/>
       <c r="AM252" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -30104,7 +30104,7 @@
         <v>1</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>0</v>
@@ -30153,7 +30153,7 @@
       </c>
       <c r="Z22" s="7" t="inlineStr">
         <is>
-          <t>Rusty Jab — Attack 3.</t>
+          <t>Rusty Jab — Attack 2, Pierce 2.</t>
         </is>
       </c>
       <c r="AA22" s="7" t="inlineStr">
@@ -30173,7 +30173,7 @@
       </c>
       <c r="AD22" s="7" t="inlineStr">
         <is>
-          <t>Dirty Stab — Attack 5, Stab. Disengage.</t>
+          <t>Dirty Stab — Attack 4, Stab. Disengage.</t>
         </is>
       </c>
       <c r="AE22" s="7" t="n">
@@ -30284,7 +30284,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="7" t="n">
         <v>5</v>
@@ -30329,7 +30329,7 @@
       </c>
       <c r="AA23" s="7" t="inlineStr">
         <is>
-          <t>Aimed Shot — Ranged Attack 4 if the target has no Guard; otherwise Ranged Attack 3.</t>
+          <t>Aimed Shot — Ranged Attack 3, Pierce 2</t>
         </is>
       </c>
       <c r="AB23" s="7" t="inlineStr">
@@ -30595,7 +30595,7 @@
         </is>
       </c>
       <c r="F25" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -30620,7 +30620,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="7" t="n">
         <v>0</v>
@@ -30661,22 +30661,22 @@
       </c>
       <c r="Y25" s="7" t="inlineStr">
         <is>
-          <t>Hex Bolt — Ranged Magic Attack 2.</t>
+          <t>Hex Bolt — Ranged Attack 3.</t>
         </is>
       </c>
       <c r="Z25" s="7" t="inlineStr">
         <is>
-          <t>Crackling Hex — Ranged Magic Attack 3.</t>
+          <t>Crackling Hex — Ranged Attack 4.</t>
         </is>
       </c>
       <c r="AA25" s="7" t="inlineStr">
         <is>
-          <t>Jinx Guard — Remove 2 Guard from the target; if it has no Guard, Ranged Magic Attack 2 instead.</t>
+          <t>Jinx Guard — Attack 3, Sunder 2</t>
         </is>
       </c>
       <c r="AB25" s="7" t="inlineStr">
         <is>
-          <t>Scurrying Ward — Move 5 ft. One ally within 30 ft gains 2 Guard.</t>
+          <t>Scurrying Ward — One ally within 30 ft gains 5 Guard. While this Guard remains, any creature that hits the ally with a melee attack is lashed by the shield and suffers Attack 3.</t>
         </is>
       </c>
       <c r="AC25" s="7" t="inlineStr">
@@ -30686,7 +30686,7 @@
       </c>
       <c r="AD25" s="7" t="inlineStr">
         <is>
-          <t>Hex Burst — Ranged Magic Attack 5. If this deals a Wound, the target discards 1 random card from hand.</t>
+          <t>Hex Burst — Ranged Magic Attack 5, Shatter. If this deals a Wound, the target discards 1 random card from hand.</t>
         </is>
       </c>
       <c r="AE25" s="7" t="n">
@@ -31130,7 +31130,7 @@
         <v>1</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="M28" s="7" t="n">
         <v>0</v>
@@ -31139,16 +31139,16 @@
         <v>1</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S28" s="7" t="n">
         <v>2</v>
@@ -31189,7 +31189,7 @@
       </c>
       <c r="AB28" s="7" t="inlineStr">
         <is>
-          <t>Ambush Blow — Attack 5 if the target has no Guard; otherwise Attack 4.</t>
+          <t>Ambush Blow — Attack 4, Overwhelm</t>
         </is>
       </c>
       <c r="AC28" s="7" t="inlineStr">
@@ -34541,7 +34541,9 @@
       <c r="AI2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ2" s="7" t="str"/>
+      <c r="AJ2" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK2" s="7" t="n">
         <v>0</v>
       </c>
@@ -34686,7 +34688,9 @@
       <c r="AI3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ3" s="7" t="str"/>
+      <c r="AJ3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK3" s="7" t="n">
         <v>0</v>
       </c>
@@ -34831,7 +34835,9 @@
       <c r="AI4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ4" s="7" t="str"/>
+      <c r="AJ4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK4" s="7" t="n">
         <v>0</v>
       </c>
@@ -34976,7 +34982,9 @@
       <c r="AI5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ5" s="7" t="str"/>
+      <c r="AJ5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK5" s="7" t="n">
         <v>0</v>
       </c>
@@ -35121,7 +35129,9 @@
       <c r="AI6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ6" s="7" t="str"/>
+      <c r="AJ6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK6" s="7" t="n">
         <v>0</v>
       </c>
@@ -35266,7 +35276,9 @@
       <c r="AI7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ7" s="7" t="str"/>
+      <c r="AJ7" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK7" s="7" t="n">
         <v>0</v>
       </c>
@@ -35411,7 +35423,9 @@
       <c r="AI8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ8" s="7" t="str"/>
+      <c r="AJ8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK8" s="7" t="n">
         <v>0</v>
       </c>
@@ -35556,7 +35570,9 @@
       <c r="AI9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ9" s="7" t="str"/>
+      <c r="AJ9" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK9" s="7" t="n">
         <v>0</v>
       </c>
@@ -35701,7 +35717,9 @@
       <c r="AI10" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ10" s="7" t="str"/>
+      <c r="AJ10" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK10" s="7" t="n">
         <v>0</v>
       </c>
@@ -35846,7 +35864,9 @@
       <c r="AI11" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ11" s="7" t="str"/>
+      <c r="AJ11" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK11" s="7" t="n">
         <v>0</v>
       </c>
@@ -40923,7 +40943,9 @@
       <c r="AI44" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ44" s="7" t="str"/>
+      <c r="AJ44" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK44" s="7" t="n">
         <v>0</v>
       </c>
@@ -41068,7 +41090,9 @@
       <c r="AI45" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ45" s="7" t="str"/>
+      <c r="AJ45" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK45" s="7" t="n">
         <v>0</v>
       </c>
@@ -41213,7 +41237,9 @@
       <c r="AI46" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ46" s="7" t="str"/>
+      <c r="AJ46" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK46" s="7" t="n">
         <v>0</v>
       </c>
@@ -41358,7 +41384,9 @@
       <c r="AI47" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ47" s="7" t="str"/>
+      <c r="AJ47" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK47" s="7" t="n">
         <v>0</v>
       </c>
@@ -41503,7 +41531,9 @@
       <c r="AI48" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ48" s="7" t="str"/>
+      <c r="AJ48" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK48" s="7" t="n">
         <v>0</v>
       </c>
@@ -41648,7 +41678,9 @@
       <c r="AI49" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AJ49" s="7" t="str"/>
+      <c r="AJ49" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK49" s="7" t="n">
         <v>0</v>
       </c>
@@ -48024,10 +48056,16 @@
           <t>None</t>
         </is>
       </c>
+      <c r="AJ41" t="n">
+        <v>0</v>
+      </c>
       <c r="AK41" t="inlineStr">
         <is>
           <t>None</t>
         </is>
+      </c>
+      <c r="AL41" t="n">
+        <v>0</v>
       </c>
       <c r="AM41" t="inlineStr">
         <is>
@@ -54306,13 +54344,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ2" s="7" t="str"/>
+      <c r="AJ2" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL2" s="7" t="str"/>
+      <c r="AL2" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM2" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -54451,13 +54493,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ3" s="7" t="str"/>
+      <c r="AJ3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK3" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL3" s="7" t="str"/>
+      <c r="AL3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM3" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -54596,13 +54642,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ4" s="7" t="str"/>
+      <c r="AJ4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK4" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL4" s="7" t="str"/>
+      <c r="AL4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM4" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -54741,13 +54791,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ5" s="7" t="str"/>
+      <c r="AJ5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK5" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL5" s="7" t="str"/>
+      <c r="AL5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM5" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -54886,13 +54940,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ6" s="7" t="str"/>
+      <c r="AJ6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK6" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL6" s="7" t="str"/>
+      <c r="AL6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM6" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -55031,13 +55089,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ7" s="7" t="str"/>
+      <c r="AJ7" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK7" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL7" s="7" t="str"/>
+      <c r="AL7" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM7" s="7" t="inlineStr">
         <is>
           <t>None</t>
@@ -55178,13 +55240,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="AJ8" s="7" t="str"/>
+      <c r="AJ8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AK8" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AL8" s="7" t="str"/>
+      <c r="AL8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="AM8" s="7" t="inlineStr">
         <is>
           <t>None</t>

</xml_diff>